<commit_message>
docs: embeber capturas de pantalla en columna Evidencia del xlsx
</commit_message>
<xml_diff>
--- a/docs/plantillas-llenas/Casos_de_Prueba.xlsx
+++ b/docs/plantillas-llenas/Casos_de_Prueba.xlsx
@@ -616,7 +616,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -665,7 +665,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -678,6 +678,1211 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId27"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId32"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId33"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId34"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId35"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId36"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId37"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId46"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId47"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3048000" cy="1390650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId48"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -918,7 +2123,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="9"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -973,7 +2178,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="90" customHeight="1">
+    <row r="2" ht="115" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
           <t>CP-LOG-01</t>
@@ -1015,13 +2220,9 @@
         </is>
       </c>
       <c r="I2" s="36" t="inlineStr"/>
-      <c r="J2" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="90" customHeight="1">
+      <c r="J2" s="37" t="inlineStr"/>
+    </row>
+    <row r="3" ht="115" customHeight="1">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>CP-LOG-02</t>
@@ -1063,13 +2264,9 @@
         </is>
       </c>
       <c r="I3" s="36" t="inlineStr"/>
-      <c r="J3" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="90" customHeight="1">
+      <c r="J3" s="37" t="inlineStr"/>
+    </row>
+    <row r="4" ht="115" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
           <t>CP-LOG-03</t>
@@ -1111,13 +2308,9 @@
         </is>
       </c>
       <c r="I4" s="36" t="inlineStr"/>
-      <c r="J4" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="90" customHeight="1">
+      <c r="J4" s="37" t="inlineStr"/>
+    </row>
+    <row r="5" ht="115" customHeight="1">
       <c r="A5" s="31" t="inlineStr">
         <is>
           <t>CP-LOG-04</t>
@@ -1159,13 +2352,9 @@
         </is>
       </c>
       <c r="I5" s="36" t="inlineStr"/>
-      <c r="J5" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="90" customHeight="1">
+      <c r="J5" s="37" t="inlineStr"/>
+    </row>
+    <row r="6" ht="115" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
         <is>
           <t>CP-LOG-05</t>
@@ -1207,13 +2396,9 @@
         </is>
       </c>
       <c r="I6" s="36" t="inlineStr"/>
-      <c r="J6" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="90" customHeight="1">
+      <c r="J6" s="37" t="inlineStr"/>
+    </row>
+    <row r="7" ht="115" customHeight="1">
       <c r="A7" s="31" t="inlineStr">
         <is>
           <t>CP-REG-01</t>
@@ -1255,13 +2440,9 @@
         </is>
       </c>
       <c r="I7" s="36" t="inlineStr"/>
-      <c r="J7" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="90" customHeight="1">
+      <c r="J7" s="37" t="inlineStr"/>
+    </row>
+    <row r="8" ht="115" customHeight="1">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>CP-REG-02</t>
@@ -1303,13 +2484,9 @@
         </is>
       </c>
       <c r="I8" s="36" t="inlineStr"/>
-      <c r="J8" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="90" customHeight="1">
+      <c r="J8" s="37" t="inlineStr"/>
+    </row>
+    <row r="9" ht="115" customHeight="1">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>CP-REG-03</t>
@@ -1351,13 +2528,9 @@
         </is>
       </c>
       <c r="I9" s="36" t="inlineStr"/>
-      <c r="J9" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="90" customHeight="1">
+      <c r="J9" s="37" t="inlineStr"/>
+    </row>
+    <row r="10" ht="115" customHeight="1">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>CP-REG-04</t>
@@ -1399,13 +2572,9 @@
         </is>
       </c>
       <c r="I10" s="36" t="inlineStr"/>
-      <c r="J10" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="90" customHeight="1">
+      <c r="J10" s="37" t="inlineStr"/>
+    </row>
+    <row r="11" ht="115" customHeight="1">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>CP-REG-05</t>
@@ -1447,13 +2616,9 @@
         </is>
       </c>
       <c r="I11" s="36" t="inlineStr"/>
-      <c r="J11" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="90" customHeight="1">
+      <c r="J11" s="37" t="inlineStr"/>
+    </row>
+    <row r="12" ht="115" customHeight="1">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>CP-REG-06</t>
@@ -1495,13 +2660,9 @@
         </is>
       </c>
       <c r="I12" s="36" t="inlineStr"/>
-      <c r="J12" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="90" customHeight="1">
+      <c r="J12" s="37" t="inlineStr"/>
+    </row>
+    <row r="13" ht="115" customHeight="1">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>CP-REG-07</t>
@@ -1543,13 +2704,9 @@
         </is>
       </c>
       <c r="I13" s="36" t="inlineStr"/>
-      <c r="J13" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="90" customHeight="1">
+      <c r="J13" s="37" t="inlineStr"/>
+    </row>
+    <row r="14" ht="115" customHeight="1">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>CP-REG-08</t>
@@ -1591,13 +2748,9 @@
         </is>
       </c>
       <c r="I14" s="36" t="inlineStr"/>
-      <c r="J14" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="90" customHeight="1">
+      <c r="J14" s="37" t="inlineStr"/>
+    </row>
+    <row r="15" ht="115" customHeight="1">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>CP-PROT-01</t>
@@ -1639,13 +2792,9 @@
         </is>
       </c>
       <c r="I15" s="36" t="inlineStr"/>
-      <c r="J15" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="90" customHeight="1">
+      <c r="J15" s="37" t="inlineStr"/>
+    </row>
+    <row r="16" ht="115" customHeight="1">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>CP-PROT-02</t>
@@ -1687,13 +2836,9 @@
         </is>
       </c>
       <c r="I16" s="36" t="inlineStr"/>
-      <c r="J16" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="90" customHeight="1">
+      <c r="J16" s="37" t="inlineStr"/>
+    </row>
+    <row r="17" ht="115" customHeight="1">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>CP-CLI-01</t>
@@ -1735,13 +2880,9 @@
         </is>
       </c>
       <c r="I17" s="36" t="inlineStr"/>
-      <c r="J17" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="90" customHeight="1">
+      <c r="J17" s="37" t="inlineStr"/>
+    </row>
+    <row r="18" ht="115" customHeight="1">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>CP-CLI-02</t>
@@ -1783,13 +2924,9 @@
         </is>
       </c>
       <c r="I18" s="36" t="inlineStr"/>
-      <c r="J18" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="90" customHeight="1">
+      <c r="J18" s="37" t="inlineStr"/>
+    </row>
+    <row r="19" ht="115" customHeight="1">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>CP-CLI-03</t>
@@ -1831,13 +2968,9 @@
         </is>
       </c>
       <c r="I19" s="36" t="inlineStr"/>
-      <c r="J19" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="90" customHeight="1">
+      <c r="J19" s="37" t="inlineStr"/>
+    </row>
+    <row r="20" ht="115" customHeight="1">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>CP-CLI-04</t>
@@ -1879,13 +3012,9 @@
         </is>
       </c>
       <c r="I20" s="36" t="inlineStr"/>
-      <c r="J20" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="90" customHeight="1">
+      <c r="J20" s="37" t="inlineStr"/>
+    </row>
+    <row r="21" ht="115" customHeight="1">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>CP-CLI-05</t>
@@ -1927,13 +3056,9 @@
         </is>
       </c>
       <c r="I21" s="36" t="inlineStr"/>
-      <c r="J21" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="90" customHeight="1">
+      <c r="J21" s="37" t="inlineStr"/>
+    </row>
+    <row r="22" ht="115" customHeight="1">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>CP-CLI-06</t>
@@ -1975,13 +3100,9 @@
         </is>
       </c>
       <c r="I22" s="36" t="inlineStr"/>
-      <c r="J22" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="90" customHeight="1">
+      <c r="J22" s="37" t="inlineStr"/>
+    </row>
+    <row r="23" ht="115" customHeight="1">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>CP-CLI-07</t>
@@ -2023,13 +3144,9 @@
         </is>
       </c>
       <c r="I23" s="36" t="inlineStr"/>
-      <c r="J23" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="90" customHeight="1">
+      <c r="J23" s="37" t="inlineStr"/>
+    </row>
+    <row r="24" ht="115" customHeight="1">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>CP-LIST-01</t>
@@ -2071,13 +3188,9 @@
         </is>
       </c>
       <c r="I24" s="36" t="inlineStr"/>
-      <c r="J24" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="90" customHeight="1">
+      <c r="J24" s="37" t="inlineStr"/>
+    </row>
+    <row r="25" ht="115" customHeight="1">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>CP-LIST-02</t>
@@ -2119,13 +3232,9 @@
         </is>
       </c>
       <c r="I25" s="36" t="inlineStr"/>
-      <c r="J25" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="90" customHeight="1">
+      <c r="J25" s="37" t="inlineStr"/>
+    </row>
+    <row r="26" ht="115" customHeight="1">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>CP-LIST-03</t>
@@ -2167,13 +3276,9 @@
         </is>
       </c>
       <c r="I26" s="36" t="inlineStr"/>
-      <c r="J26" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="90" customHeight="1">
+      <c r="J26" s="37" t="inlineStr"/>
+    </row>
+    <row r="27" ht="115" customHeight="1">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>CP-LIST-04</t>
@@ -2215,13 +3320,9 @@
         </is>
       </c>
       <c r="I27" s="36" t="inlineStr"/>
-      <c r="J27" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="90" customHeight="1">
+      <c r="J27" s="37" t="inlineStr"/>
+    </row>
+    <row r="28" ht="115" customHeight="1">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>CP-LIST-05</t>
@@ -2263,13 +3364,9 @@
         </is>
       </c>
       <c r="I28" s="36" t="inlineStr"/>
-      <c r="J28" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="90" customHeight="1">
+      <c r="J28" s="37" t="inlineStr"/>
+    </row>
+    <row r="29" ht="115" customHeight="1">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>CP-LIST-06</t>
@@ -2311,13 +3408,9 @@
         </is>
       </c>
       <c r="I29" s="36" t="inlineStr"/>
-      <c r="J29" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="90" customHeight="1">
+      <c r="J29" s="37" t="inlineStr"/>
+    </row>
+    <row r="30" ht="115" customHeight="1">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>CP-LIST-07</t>
@@ -2359,13 +3452,9 @@
         </is>
       </c>
       <c r="I30" s="36" t="inlineStr"/>
-      <c r="J30" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="90" customHeight="1">
+      <c r="J30" s="37" t="inlineStr"/>
+    </row>
+    <row r="31" ht="115" customHeight="1">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>CP-LIST-08</t>
@@ -2407,13 +3496,9 @@
         </is>
       </c>
       <c r="I31" s="36" t="inlineStr"/>
-      <c r="J31" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="90" customHeight="1">
+      <c r="J31" s="37" t="inlineStr"/>
+    </row>
+    <row r="32" ht="115" customHeight="1">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>CP-DEL-01</t>
@@ -2455,13 +3540,9 @@
         </is>
       </c>
       <c r="I32" s="36" t="inlineStr"/>
-      <c r="J32" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="90" customHeight="1">
+      <c r="J32" s="37" t="inlineStr"/>
+    </row>
+    <row r="33" ht="115" customHeight="1">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>CP-DEL-02</t>
@@ -2503,13 +3584,9 @@
         </is>
       </c>
       <c r="I33" s="36" t="inlineStr"/>
-      <c r="J33" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="90" customHeight="1">
+      <c r="J33" s="37" t="inlineStr"/>
+    </row>
+    <row r="34" ht="115" customHeight="1">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>CP-DEL-03</t>
@@ -2551,13 +3628,9 @@
         </is>
       </c>
       <c r="I34" s="36" t="inlineStr"/>
-      <c r="J34" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="90" customHeight="1">
+      <c r="J34" s="37" t="inlineStr"/>
+    </row>
+    <row r="35" ht="115" customHeight="1">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>CP-DEL-04</t>
@@ -2599,13 +3672,9 @@
         </is>
       </c>
       <c r="I35" s="36" t="inlineStr"/>
-      <c r="J35" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="90" customHeight="1">
+      <c r="J35" s="37" t="inlineStr"/>
+    </row>
+    <row r="36" ht="115" customHeight="1">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>CP-DEL-05</t>
@@ -2647,13 +3716,9 @@
         </is>
       </c>
       <c r="I36" s="36" t="inlineStr"/>
-      <c r="J36" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="90" customHeight="1">
+      <c r="J36" s="37" t="inlineStr"/>
+    </row>
+    <row r="37" ht="115" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>CP-KPI-01</t>
@@ -2695,13 +3760,9 @@
         </is>
       </c>
       <c r="I37" s="36" t="inlineStr"/>
-      <c r="J37" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="90" customHeight="1">
+      <c r="J37" s="37" t="inlineStr"/>
+    </row>
+    <row r="38" ht="115" customHeight="1">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>CP-KPI-02</t>
@@ -2743,13 +3804,9 @@
         </is>
       </c>
       <c r="I38" s="36" t="inlineStr"/>
-      <c r="J38" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="90" customHeight="1">
+      <c r="J38" s="37" t="inlineStr"/>
+    </row>
+    <row r="39" ht="115" customHeight="1">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>CP-KPI-03</t>
@@ -2791,13 +3848,9 @@
         </is>
       </c>
       <c r="I39" s="36" t="inlineStr"/>
-      <c r="J39" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="90" customHeight="1">
+      <c r="J39" s="37" t="inlineStr"/>
+    </row>
+    <row r="40" ht="115" customHeight="1">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>CP-KPI-04</t>
@@ -2839,13 +3892,9 @@
         </is>
       </c>
       <c r="I40" s="36" t="inlineStr"/>
-      <c r="J40" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="90" customHeight="1">
+      <c r="J40" s="37" t="inlineStr"/>
+    </row>
+    <row r="41" ht="115" customHeight="1">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>CP-KPI-05</t>
@@ -2887,13 +3936,9 @@
         </is>
       </c>
       <c r="I41" s="36" t="inlineStr"/>
-      <c r="J41" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="90" customHeight="1">
+      <c r="J41" s="37" t="inlineStr"/>
+    </row>
+    <row r="42" ht="115" customHeight="1">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>CP-CHART-01</t>
@@ -2935,13 +3980,9 @@
         </is>
       </c>
       <c r="I42" s="36" t="inlineStr"/>
-      <c r="J42" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="90" customHeight="1">
+      <c r="J42" s="37" t="inlineStr"/>
+    </row>
+    <row r="43" ht="115" customHeight="1">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>CP-CHART-02</t>
@@ -2983,13 +4024,9 @@
         </is>
       </c>
       <c r="I43" s="36" t="inlineStr"/>
-      <c r="J43" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="90" customHeight="1">
+      <c r="J43" s="37" t="inlineStr"/>
+    </row>
+    <row r="44" ht="115" customHeight="1">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>CP-CHART-03</t>
@@ -3031,13 +4068,9 @@
         </is>
       </c>
       <c r="I44" s="36" t="inlineStr"/>
-      <c r="J44" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="90" customHeight="1">
+      <c r="J44" s="37" t="inlineStr"/>
+    </row>
+    <row r="45" ht="115" customHeight="1">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>CP-CHART-04</t>
@@ -3079,13 +4112,9 @@
         </is>
       </c>
       <c r="I45" s="36" t="inlineStr"/>
-      <c r="J45" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="90" customHeight="1">
+      <c r="J45" s="37" t="inlineStr"/>
+    </row>
+    <row r="46" ht="115" customHeight="1">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>CP-ATTEN-01</t>
@@ -3127,13 +4156,9 @@
         </is>
       </c>
       <c r="I46" s="36" t="inlineStr"/>
-      <c r="J46" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="90" customHeight="1">
+      <c r="J46" s="37" t="inlineStr"/>
+    </row>
+    <row r="47" ht="115" customHeight="1">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>CP-ATTEN-02</t>
@@ -3175,13 +4200,9 @@
         </is>
       </c>
       <c r="I47" s="36" t="inlineStr"/>
-      <c r="J47" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="90" customHeight="1">
+      <c r="J47" s="37" t="inlineStr"/>
+    </row>
+    <row r="48" ht="115" customHeight="1">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>CP-ATTEN-03</t>
@@ -3223,13 +4244,9 @@
         </is>
       </c>
       <c r="I48" s="36" t="inlineStr"/>
-      <c r="J48" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="90" customHeight="1">
+      <c r="J48" s="37" t="inlineStr"/>
+    </row>
+    <row r="49" ht="115" customHeight="1">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>CP-ATTEN-04</t>
@@ -3271,11 +4288,7 @@
         </is>
       </c>
       <c r="I49" s="36" t="inlineStr"/>
-      <c r="J49" s="37" t="inlineStr">
-        <is>
-          <t>Captura de pantalla</t>
-        </is>
-      </c>
+      <c r="J49" s="37" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J6"/>
@@ -3293,6 +4306,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix(docs): re-etiquetar pruebas de registro (CP-REG) como Sprint 1, no Sprint 2
</commit_message>
<xml_diff>
--- a/docs/plantillas-llenas/Casos_de_Prueba.xlsx
+++ b/docs/plantillas-llenas/Casos_de_Prueba.xlsx
@@ -700,6 +700,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -725,6 +728,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -750,6 +756,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -775,6 +784,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -800,6 +812,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -825,6 +840,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -850,6 +868,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -875,6 +896,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -900,6 +924,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -925,6 +952,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -950,6 +980,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -975,6 +1008,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1000,6 +1036,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1025,6 +1064,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1050,6 +1092,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1075,6 +1120,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1100,6 +1148,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1125,6 +1176,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1150,6 +1204,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1175,6 +1232,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1200,6 +1260,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1225,6 +1288,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1250,6 +1316,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1275,6 +1344,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1300,6 +1372,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1325,6 +1400,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1350,6 +1428,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1375,6 +1456,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1400,6 +1484,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1425,6 +1512,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1450,6 +1540,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1475,6 +1568,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1500,6 +1596,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1525,6 +1624,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1550,6 +1652,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1575,6 +1680,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1600,6 +1708,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1625,6 +1736,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1650,6 +1764,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1675,6 +1792,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1700,6 +1820,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1725,6 +1848,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1750,6 +1876,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1775,6 +1904,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1800,6 +1932,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1825,6 +1960,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1850,6 +1988,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1875,6 +2016,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2436,7 +2580,7 @@
       </c>
       <c r="H7" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="I7" s="36" t="inlineStr"/>
@@ -2480,7 +2624,7 @@
       </c>
       <c r="H8" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="I8" s="36" t="inlineStr"/>
@@ -2524,7 +2668,7 @@
       </c>
       <c r="H9" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="I9" s="36" t="inlineStr"/>
@@ -2568,7 +2712,7 @@
       </c>
       <c r="H10" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="I10" s="36" t="inlineStr"/>
@@ -2612,7 +2756,7 @@
       </c>
       <c r="H11" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="I11" s="36" t="inlineStr"/>
@@ -2656,7 +2800,7 @@
       </c>
       <c r="H12" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="I12" s="36" t="inlineStr"/>
@@ -2700,7 +2844,7 @@
       </c>
       <c r="H13" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="I13" s="36" t="inlineStr"/>
@@ -2744,7 +2888,7 @@
       </c>
       <c r="H14" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="I14" s="36" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: ordenar casos de prueba por sprint en el xlsx
</commit_message>
<xml_diff>
--- a/docs/plantillas-llenas/Casos_de_Prueba.xlsx
+++ b/docs/plantillas-llenas/Casos_de_Prueba.xlsx
@@ -700,9 +700,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -728,9 +725,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -756,9 +750,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -784,9 +775,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -812,9 +800,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -840,9 +825,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -868,9 +850,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -896,9 +875,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -924,9 +900,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -952,9 +925,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -980,9 +950,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1008,9 +975,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1036,9 +1000,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1064,9 +1025,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1092,9 +1050,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1120,9 +1075,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1148,9 +1100,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1176,9 +1125,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1204,9 +1150,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1232,9 +1175,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1260,9 +1200,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1288,9 +1225,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1316,9 +1250,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1344,9 +1275,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1372,9 +1300,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1400,9 +1325,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1428,9 +1350,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1456,9 +1375,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1484,9 +1400,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1512,9 +1425,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1540,9 +1450,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1568,9 +1475,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1596,9 +1500,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1624,9 +1525,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1652,9 +1550,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1680,9 +1575,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1708,9 +1600,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1736,9 +1625,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1764,9 +1650,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1792,9 +1675,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1820,9 +1700,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1848,9 +1725,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1876,9 +1750,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1904,9 +1775,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1932,9 +1800,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1960,9 +1825,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1988,9 +1850,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2016,9 +1875,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2325,32 +2181,32 @@
     <row r="2" ht="115" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>CP-LOG-01</t>
+          <t>CP-REG-01</t>
         </is>
       </c>
       <c r="B2" s="32" t="inlineStr">
         <is>
-          <t>Validación de correo en inicio de sesión</t>
+          <t>Validación de datos obligatorios</t>
         </is>
       </c>
       <c r="C2" s="33" t="inlineStr">
         <is>
-          <t>El usuario intenta iniciar sesión con un correo mal escrito</t>
+          <t>El usuario intenta registrarse sin proporcionar la información básica</t>
         </is>
       </c>
       <c r="D2" s="33" t="inlineStr">
         <is>
-          <t>Me encuentro en la pantalla de inicio de sesión de la plataforma</t>
+          <t>Me encuentro en la pantalla de crear una cuenta nueva</t>
         </is>
       </c>
       <c r="E2" s="33" t="inlineStr">
         <is>
-          <t>Escribo un correo sin usar el formato correcto (por ejemplo, omitiendo el @) y paso al campo de la contraseña</t>
+          <t>Hago clic en el botón 'Registrarse' sin haber llenado ningún dato</t>
         </is>
       </c>
       <c r="F2" s="32" t="inlineStr">
         <is>
-          <t>Aparece un mensaje debajo del campo indicando: 'Ingresa una dirección de correo válida'</t>
+          <t>Todos los campos vacíos se pintan de rojo y muestran indicando: 'Este campo es obligatorio'</t>
         </is>
       </c>
       <c r="G2" s="34" t="inlineStr">
@@ -2360,41 +2216,41 @@
       </c>
       <c r="H2" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-      <c r="I2" s="36" t="inlineStr"/>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="I2" s="36" t="n"/>
       <c r="J2" s="37" t="inlineStr"/>
     </row>
     <row r="3" ht="115" customHeight="1">
       <c r="A3" s="31" t="inlineStr">
         <is>
-          <t>CP-LOG-02</t>
+          <t>CP-REG-02</t>
         </is>
       </c>
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>Credenciales incorrectas al iniciar sesión</t>
+          <t>Formato de correo en registro</t>
         </is>
       </c>
       <c r="C3" s="33" t="inlineStr">
         <is>
-          <t>El usuario ingresa datos que no coinciden con una cuenta existente</t>
+          <t>El usuario escribe mal su correo durante el proceso de registro</t>
         </is>
       </c>
       <c r="D3" s="33" t="inlineStr">
         <is>
-          <t>Me encuentro en la pantalla de inicio de sesión</t>
+          <t>Me encuentro llenando el formulario de registro</t>
         </is>
       </c>
       <c r="E3" s="33" t="inlineStr">
         <is>
-          <t>Ingreso un correo o una contraseña equivocados y hago clic en 'Iniciar sesión'</t>
+          <t>Escribo mi correo de forma incorrecta (ej. sin el @) y trato de crear la cuenta</t>
         </is>
       </c>
       <c r="F3" s="32" t="inlineStr">
         <is>
-          <t>Aparece una alerta que dice: 'El correo o la contraseña son incorrectos', sin revelar explícitamente a un extraño cuál de los dos falló</t>
+          <t>El sistema me impide continuar y me alerta de inmediato: 'Ingresa una dirección de correo válida'</t>
         </is>
       </c>
       <c r="G3" s="34" t="inlineStr">
@@ -2404,41 +2260,41 @@
       </c>
       <c r="H3" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-      <c r="I3" s="36" t="inlineStr"/>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="I3" s="36" t="n"/>
       <c r="J3" s="37" t="inlineStr"/>
     </row>
     <row r="4" ht="115" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
-          <t>CP-LOG-03</t>
+          <t>CP-REG-03</t>
         </is>
       </c>
       <c r="B4" s="32" t="inlineStr">
         <is>
-          <t>Inicio de sesión exitoso</t>
+          <t>Validación de números en teléfono</t>
         </is>
       </c>
       <c r="C4" s="33" t="inlineStr">
         <is>
-          <t>El usuario ingresa a la plataforma correctamente con sus datos validados</t>
+          <t>El usuario intenta introducir letras en su número de contacto</t>
         </is>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
-          <t>Me encuentro en la pantalla de inicio de sesión y tengo una cuenta válida</t>
+          <t>Me encuentro llenando el número de teléfono en el formulario de registro</t>
         </is>
       </c>
       <c r="E4" s="33" t="inlineStr">
         <is>
-          <t>Ingreso mi correo electrónico y contraseña correctos, y hago clic en 'Iniciar sesión'</t>
+          <t>Empiezo a teclear letras y caracteres especiales en lugar de números</t>
         </is>
       </c>
       <c r="F4" s="32" t="inlineStr">
         <is>
-          <t>Ingreso exitosamente al sistema y puedo ver mi pantalla principal (Panel de Control)</t>
+          <t>El campo no me permite escribir esos caracteres; solo recibe números y me obliga a poner exactamente 10 dígitos</t>
         </is>
       </c>
       <c r="G4" s="34" t="inlineStr">
@@ -2448,41 +2304,41 @@
       </c>
       <c r="H4" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-      <c r="I4" s="36" t="inlineStr"/>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="I4" s="36" t="n"/>
       <c r="J4" s="37" t="inlineStr"/>
     </row>
     <row r="5" ht="115" customHeight="1">
       <c r="A5" s="31" t="inlineStr">
         <is>
-          <t>CP-LOG-04</t>
+          <t>CP-REG-04</t>
         </is>
       </c>
       <c r="B5" s="32" t="inlineStr">
         <is>
-          <t>Enlace de olvidar contraseña</t>
+          <t>Confirmación de contraseñas</t>
         </is>
       </c>
       <c r="C5" s="33" t="inlineStr">
         <is>
-          <t>El usuario intenta recuperar su clave haciendo clic en el enlace</t>
+          <t>El usuario escribe contraseñas diferentes por accidente</t>
         </is>
       </c>
       <c r="D5" s="33" t="inlineStr">
         <is>
-          <t>Me encuentro en la pantalla de inicio de sesión y no recuerdo mi clave</t>
+          <t>Me encuentro en la sección de contraseñas del formulario de registro</t>
         </is>
       </c>
       <c r="E5" s="33" t="inlineStr">
         <is>
-          <t>Hago clic en el botón o enlace que dice '¿Olvidaste tu contraseña?'</t>
+          <t>Escribo una clave inicial y abajo en la confirmación pongo una distinta, luego hago clic en 'Registrarse'</t>
         </is>
       </c>
       <c r="F5" s="32" t="inlineStr">
         <is>
-          <t>El sistema me muestra un mensaje informativo diciendo que 'Esta función estará disponible próximamente'</t>
+          <t>El sistema me impide finalizar y muestra un mensaje rojo alertando: 'Las contraseñas no coinciden'</t>
         </is>
       </c>
       <c r="G5" s="34" t="inlineStr">
@@ -2492,41 +2348,41 @@
       </c>
       <c r="H5" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-      <c r="I5" s="36" t="inlineStr"/>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="I5" s="36" t="n"/>
       <c r="J5" s="37" t="inlineStr"/>
     </row>
     <row r="6" ht="115" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
         <is>
-          <t>CP-LOG-05</t>
+          <t>CP-REG-05</t>
         </is>
       </c>
       <c r="B6" s="32" t="inlineStr">
         <is>
-          <t>Mostrar y ocultar contraseña</t>
+          <t>Bloqueo de doble clic al registrar</t>
         </is>
       </c>
       <c r="C6" s="33" t="inlineStr">
         <is>
-          <t>El usuario quiere comprobar si escribió bien su contraseña visualizando los caracteres</t>
+          <t>El usuario presiona varias veces seguidas el botón de registrarse</t>
         </is>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
-          <t>Me encuentro en la pantalla de inicio de sesión escribiendo mi contraseña</t>
+          <t>Llené correctamente todos mis datos para confirmar la cuenta</t>
         </is>
       </c>
       <c r="E6" s="33" t="inlineStr">
         <is>
-          <t>Hago clic en el pequeño icono del ojo al lado del campo de contraseña</t>
+          <t>Hago clic rápida y repetidamente en el botón principal de 'Registrarse'</t>
         </is>
       </c>
       <c r="F6" s="32" t="inlineStr">
         <is>
-          <t>Los puntos se convierten en texto visible para poder leer la contraseña. Si vuelvo a hacer clic, se ocultan de nuevo</t>
+          <t>El botón cambia a decir 'Creando cuenta...' y no me deja seguir haciendo clics, evitando que la cuenta se cree dos veces</t>
         </is>
       </c>
       <c r="G6" s="34" t="inlineStr">
@@ -2536,41 +2392,41 @@
       </c>
       <c r="H6" s="35" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-      <c r="I6" s="36" t="inlineStr"/>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="I6" s="36" t="n"/>
       <c r="J6" s="37" t="inlineStr"/>
     </row>
     <row r="7" ht="115" customHeight="1">
       <c r="A7" s="31" t="inlineStr">
         <is>
-          <t>CP-REG-01</t>
+          <t>CP-REG-06</t>
         </is>
       </c>
       <c r="B7" s="32" t="inlineStr">
         <is>
-          <t>Validación de datos obligatorios</t>
+          <t>Creación de cuenta exitosa</t>
         </is>
       </c>
       <c r="C7" s="33" t="inlineStr">
         <is>
-          <t>El usuario intenta registrarse sin proporcionar la información básica</t>
+          <t>El usuario completa todo el flujo y se le da la bienvenida</t>
         </is>
       </c>
       <c r="D7" s="33" t="inlineStr">
         <is>
-          <t>Me encuentro en la pantalla de crear una cuenta nueva</t>
+          <t>Llené todos mis datos de forma correcta y uso un correo totalmente nuevo</t>
         </is>
       </c>
       <c r="E7" s="33" t="inlineStr">
         <is>
-          <t>Hago clic en el botón 'Registrarse' sin haber llenado ningún dato</t>
+          <t>Hago clic en el botón de 'Registrarse'</t>
         </is>
       </c>
       <c r="F7" s="32" t="inlineStr">
         <is>
-          <t>Todos los campos vacíos se pintan de rojo y muestran indicando: 'Este campo es obligatorio'</t>
+          <t>El sistema me lleva a la pantalla de inicio de sesión mostrándome un aviso de éxito en verde: 'Tu cuenta ha sido creada. Bienvenido a CRM Cloud'</t>
         </is>
       </c>
       <c r="G7" s="34" t="inlineStr">
@@ -2583,38 +2439,38 @@
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="I7" s="36" t="inlineStr"/>
+      <c r="I7" s="36" t="n"/>
       <c r="J7" s="37" t="inlineStr"/>
     </row>
     <row r="8" ht="115" customHeight="1">
       <c r="A8" s="31" t="inlineStr">
         <is>
-          <t>CP-REG-02</t>
+          <t>CP-REG-07</t>
         </is>
       </c>
       <c r="B8" s="32" t="inlineStr">
         <is>
-          <t>Formato de correo en registro</t>
+          <t>Falla momentánea al registrar</t>
         </is>
       </c>
       <c r="C8" s="33" t="inlineStr">
         <is>
-          <t>El usuario escribe mal su correo durante el proceso de registro</t>
+          <t>El servicio experimenta un fallo de conexión temporal al momento en que el usuario intenta el registro</t>
         </is>
       </c>
       <c r="D8" s="33" t="inlineStr">
         <is>
-          <t>Me encuentro llenando el formulario de registro</t>
+          <t>Llené mis datos para registrarme</t>
         </is>
       </c>
       <c r="E8" s="33" t="inlineStr">
         <is>
-          <t>Escribo mi correo de forma incorrecta (ej. sin el @) y trato de crear la cuenta</t>
+          <t>Hago clic en 'Registrarse', pero ocurre un problema técnico y general en internet</t>
         </is>
       </c>
       <c r="F8" s="32" t="inlineStr">
         <is>
-          <t>El sistema me impide continuar y me alerta de inmediato: 'Ingresa una dirección de correo válida'</t>
+          <t>La plataforma no se queda congelada; sino que me avisa cortésmente: 'No fue posible crear la cuenta. Por favor intenta de nuevo más tarde'</t>
         </is>
       </c>
       <c r="G8" s="34" t="inlineStr">
@@ -2627,38 +2483,38 @@
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="I8" s="36" t="inlineStr"/>
+      <c r="I8" s="36" t="n"/>
       <c r="J8" s="37" t="inlineStr"/>
     </row>
     <row r="9" ht="115" customHeight="1">
       <c r="A9" s="31" t="inlineStr">
         <is>
-          <t>CP-REG-03</t>
+          <t>CP-REG-08</t>
         </is>
       </c>
       <c r="B9" s="32" t="inlineStr">
         <is>
-          <t>Validación de números en teléfono</t>
+          <t>Intento de usar correo registrado</t>
         </is>
       </c>
       <c r="C9" s="33" t="inlineStr">
         <is>
-          <t>El usuario intenta introducir letras en su número de contacto</t>
+          <t>El usuario se registra con un correo que ya fue usado por otra persona</t>
         </is>
       </c>
       <c r="D9" s="33" t="inlineStr">
         <is>
-          <t>Me encuentro llenando el número de teléfono en el formulario de registro</t>
+          <t>Escribo mis datos usando un correo electrónico que ya pertenece a otro usuario registrado</t>
         </is>
       </c>
       <c r="E9" s="33" t="inlineStr">
         <is>
-          <t>Empiezo a teclear letras y caracteres especiales en lugar de números</t>
+          <t>Hago clic en el botón de 'Registrarse'</t>
         </is>
       </c>
       <c r="F9" s="32" t="inlineStr">
         <is>
-          <t>El campo no me permite escribir esos caracteres; solo recibe números y me obliga a poner exactamente 10 dígitos</t>
+          <t>Recibo un mensaje claro y conciso que me advierte: 'Este correo ya tiene una cuenta registrada'</t>
         </is>
       </c>
       <c r="G9" s="34" t="inlineStr">
@@ -2671,38 +2527,38 @@
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="I9" s="36" t="inlineStr"/>
+      <c r="I9" s="36" t="n"/>
       <c r="J9" s="37" t="inlineStr"/>
     </row>
     <row r="10" ht="115" customHeight="1">
       <c r="A10" s="31" t="inlineStr">
         <is>
-          <t>CP-REG-04</t>
+          <t>CP-LOG-01</t>
         </is>
       </c>
       <c r="B10" s="32" t="inlineStr">
         <is>
-          <t>Confirmación de contraseñas</t>
+          <t>Validación de correo en inicio de sesión</t>
         </is>
       </c>
       <c r="C10" s="33" t="inlineStr">
         <is>
-          <t>El usuario escribe contraseñas diferentes por accidente</t>
+          <t>El usuario intenta iniciar sesión con un correo mal escrito</t>
         </is>
       </c>
       <c r="D10" s="33" t="inlineStr">
         <is>
-          <t>Me encuentro en la sección de contraseñas del formulario de registro</t>
+          <t>Me encuentro en la pantalla de inicio de sesión de la plataforma</t>
         </is>
       </c>
       <c r="E10" s="33" t="inlineStr">
         <is>
-          <t>Escribo una clave inicial y abajo en la confirmación pongo una distinta, luego hago clic en 'Registrarse'</t>
+          <t>Escribo un correo sin usar el formato correcto (por ejemplo, omitiendo el @) y paso al campo de la contraseña</t>
         </is>
       </c>
       <c r="F10" s="32" t="inlineStr">
         <is>
-          <t>El sistema me impide finalizar y muestra un mensaje rojo alertando: 'Las contraseñas no coinciden'</t>
+          <t>Aparece un mensaje debajo del campo indicando: 'Ingresa una dirección de correo válida'</t>
         </is>
       </c>
       <c r="G10" s="34" t="inlineStr">
@@ -2712,41 +2568,41 @@
       </c>
       <c r="H10" s="35" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I10" s="36" t="inlineStr"/>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="I10" s="36" t="n"/>
       <c r="J10" s="37" t="inlineStr"/>
     </row>
     <row r="11" ht="115" customHeight="1">
       <c r="A11" s="31" t="inlineStr">
         <is>
-          <t>CP-REG-05</t>
+          <t>CP-LOG-02</t>
         </is>
       </c>
       <c r="B11" s="32" t="inlineStr">
         <is>
-          <t>Bloqueo de doble clic al registrar</t>
+          <t>Credenciales incorrectas al iniciar sesión</t>
         </is>
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>El usuario presiona varias veces seguidas el botón de registrarse</t>
+          <t>El usuario ingresa datos que no coinciden con una cuenta existente</t>
         </is>
       </c>
       <c r="D11" s="33" t="inlineStr">
         <is>
-          <t>Llené correctamente todos mis datos para confirmar la cuenta</t>
+          <t>Me encuentro en la pantalla de inicio de sesión</t>
         </is>
       </c>
       <c r="E11" s="33" t="inlineStr">
         <is>
-          <t>Hago clic rápida y repetidamente en el botón principal de 'Registrarse'</t>
+          <t>Ingreso un correo o una contraseña equivocados y hago clic en 'Iniciar sesión'</t>
         </is>
       </c>
       <c r="F11" s="32" t="inlineStr">
         <is>
-          <t>El botón cambia a decir 'Creando cuenta...' y no me deja seguir haciendo clics, evitando que la cuenta se cree dos veces</t>
+          <t>Aparece una alerta que dice: 'El correo o la contraseña son incorrectos', sin revelar explícitamente a un extraño cuál de los dos falló</t>
         </is>
       </c>
       <c r="G11" s="34" t="inlineStr">
@@ -2756,41 +2612,41 @@
       </c>
       <c r="H11" s="35" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I11" s="36" t="inlineStr"/>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="I11" s="36" t="n"/>
       <c r="J11" s="37" t="inlineStr"/>
     </row>
     <row r="12" ht="115" customHeight="1">
       <c r="A12" s="31" t="inlineStr">
         <is>
-          <t>CP-REG-06</t>
+          <t>CP-LOG-03</t>
         </is>
       </c>
       <c r="B12" s="32" t="inlineStr">
         <is>
-          <t>Creación de cuenta exitosa</t>
+          <t>Inicio de sesión exitoso</t>
         </is>
       </c>
       <c r="C12" s="33" t="inlineStr">
         <is>
-          <t>El usuario completa todo el flujo y se le da la bienvenida</t>
+          <t>El usuario ingresa a la plataforma correctamente con sus datos validados</t>
         </is>
       </c>
       <c r="D12" s="33" t="inlineStr">
         <is>
-          <t>Llené todos mis datos de forma correcta y uso un correo totalmente nuevo</t>
+          <t>Me encuentro en la pantalla de inicio de sesión y tengo una cuenta válida</t>
         </is>
       </c>
       <c r="E12" s="33" t="inlineStr">
         <is>
-          <t>Hago clic en el botón de 'Registrarse'</t>
+          <t>Ingreso mi correo electrónico y contraseña correctos, y hago clic en 'Iniciar sesión'</t>
         </is>
       </c>
       <c r="F12" s="32" t="inlineStr">
         <is>
-          <t>El sistema me lleva a la pantalla de inicio de sesión mostrándome un aviso de éxito en verde: 'Tu cuenta ha sido creada. Bienvenido a CRM Cloud'</t>
+          <t>Ingreso exitosamente al sistema y puedo ver mi pantalla principal (Panel de Control)</t>
         </is>
       </c>
       <c r="G12" s="34" t="inlineStr">
@@ -2800,41 +2656,41 @@
       </c>
       <c r="H12" s="35" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I12" s="36" t="inlineStr"/>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="I12" s="36" t="n"/>
       <c r="J12" s="37" t="inlineStr"/>
     </row>
     <row r="13" ht="115" customHeight="1">
       <c r="A13" s="31" t="inlineStr">
         <is>
-          <t>CP-REG-07</t>
+          <t>CP-LOG-04</t>
         </is>
       </c>
       <c r="B13" s="32" t="inlineStr">
         <is>
-          <t>Falla momentánea al registrar</t>
+          <t>Enlace de olvidar contraseña</t>
         </is>
       </c>
       <c r="C13" s="33" t="inlineStr">
         <is>
-          <t>El servicio experimenta un fallo de conexión temporal al momento en que el usuario intenta el registro</t>
+          <t>El usuario intenta recuperar su clave haciendo clic en el enlace</t>
         </is>
       </c>
       <c r="D13" s="33" t="inlineStr">
         <is>
-          <t>Llené mis datos para registrarme</t>
+          <t>Me encuentro en la pantalla de inicio de sesión y no recuerdo mi clave</t>
         </is>
       </c>
       <c r="E13" s="33" t="inlineStr">
         <is>
-          <t>Hago clic en 'Registrarse', pero ocurre un problema técnico y general en internet</t>
+          <t>Hago clic en el botón o enlace que dice '¿Olvidaste tu contraseña?'</t>
         </is>
       </c>
       <c r="F13" s="32" t="inlineStr">
         <is>
-          <t>La plataforma no se queda congelada; sino que me avisa cortésmente: 'No fue posible crear la cuenta. Por favor intenta de nuevo más tarde'</t>
+          <t>El sistema me muestra un mensaje informativo diciendo que 'Esta función estará disponible próximamente'</t>
         </is>
       </c>
       <c r="G13" s="34" t="inlineStr">
@@ -2844,41 +2700,41 @@
       </c>
       <c r="H13" s="35" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I13" s="36" t="inlineStr"/>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="I13" s="36" t="n"/>
       <c r="J13" s="37" t="inlineStr"/>
     </row>
     <row r="14" ht="115" customHeight="1">
       <c r="A14" s="31" t="inlineStr">
         <is>
-          <t>CP-REG-08</t>
+          <t>CP-LOG-05</t>
         </is>
       </c>
       <c r="B14" s="32" t="inlineStr">
         <is>
-          <t>Intento de usar correo registrado</t>
+          <t>Mostrar y ocultar contraseña</t>
         </is>
       </c>
       <c r="C14" s="33" t="inlineStr">
         <is>
-          <t>El usuario se registra con un correo que ya fue usado por otra persona</t>
+          <t>El usuario quiere comprobar si escribió bien su contraseña visualizando los caracteres</t>
         </is>
       </c>
       <c r="D14" s="33" t="inlineStr">
         <is>
-          <t>Escribo mis datos usando un correo electrónico que ya pertenece a otro usuario registrado</t>
+          <t>Me encuentro en la pantalla de inicio de sesión escribiendo mi contraseña</t>
         </is>
       </c>
       <c r="E14" s="33" t="inlineStr">
         <is>
-          <t>Hago clic en el botón de 'Registrarse'</t>
+          <t>Hago clic en el pequeño icono del ojo al lado del campo de contraseña</t>
         </is>
       </c>
       <c r="F14" s="32" t="inlineStr">
         <is>
-          <t>Recibo un mensaje claro y conciso que me advierte: 'Este correo ya tiene una cuenta registrada'</t>
+          <t>Los puntos se convierten en texto visible para poder leer la contraseña. Si vuelvo a hacer clic, se ocultan de nuevo</t>
         </is>
       </c>
       <c r="G14" s="34" t="inlineStr">
@@ -2888,10 +2744,10 @@
       </c>
       <c r="H14" s="35" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I14" s="36" t="inlineStr"/>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="I14" s="36" t="n"/>
       <c r="J14" s="37" t="inlineStr"/>
     </row>
     <row r="15" ht="115" customHeight="1">
@@ -2935,7 +2791,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="I15" s="36" t="inlineStr"/>
+      <c r="I15" s="36" t="n"/>
       <c r="J15" s="37" t="inlineStr"/>
     </row>
     <row r="16" ht="115" customHeight="1">
@@ -2979,7 +2835,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="I16" s="36" t="inlineStr"/>
+      <c r="I16" s="36" t="n"/>
       <c r="J16" s="37" t="inlineStr"/>
     </row>
     <row r="17" ht="115" customHeight="1">
@@ -3023,7 +2879,7 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="I17" s="36" t="inlineStr"/>
+      <c r="I17" s="36" t="n"/>
       <c r="J17" s="37" t="inlineStr"/>
     </row>
     <row r="18" ht="115" customHeight="1">
@@ -3067,7 +2923,7 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="I18" s="36" t="inlineStr"/>
+      <c r="I18" s="36" t="n"/>
       <c r="J18" s="37" t="inlineStr"/>
     </row>
     <row r="19" ht="115" customHeight="1">
@@ -3111,7 +2967,7 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="I19" s="36" t="inlineStr"/>
+      <c r="I19" s="36" t="n"/>
       <c r="J19" s="37" t="inlineStr"/>
     </row>
     <row r="20" ht="115" customHeight="1">
@@ -3155,7 +3011,7 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="I20" s="36" t="inlineStr"/>
+      <c r="I20" s="36" t="n"/>
       <c r="J20" s="37" t="inlineStr"/>
     </row>
     <row r="21" ht="115" customHeight="1">
@@ -3199,7 +3055,7 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="I21" s="36" t="inlineStr"/>
+      <c r="I21" s="36" t="n"/>
       <c r="J21" s="37" t="inlineStr"/>
     </row>
     <row r="22" ht="115" customHeight="1">
@@ -3243,7 +3099,7 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="I22" s="36" t="inlineStr"/>
+      <c r="I22" s="36" t="n"/>
       <c r="J22" s="37" t="inlineStr"/>
     </row>
     <row r="23" ht="115" customHeight="1">
@@ -3287,7 +3143,7 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="I23" s="36" t="inlineStr"/>
+      <c r="I23" s="36" t="n"/>
       <c r="J23" s="37" t="inlineStr"/>
     </row>
     <row r="24" ht="115" customHeight="1">
@@ -3331,7 +3187,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="I24" s="36" t="inlineStr"/>
+      <c r="I24" s="36" t="n"/>
       <c r="J24" s="37" t="inlineStr"/>
     </row>
     <row r="25" ht="115" customHeight="1">
@@ -3375,7 +3231,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="I25" s="36" t="inlineStr"/>
+      <c r="I25" s="36" t="n"/>
       <c r="J25" s="37" t="inlineStr"/>
     </row>
     <row r="26" ht="115" customHeight="1">
@@ -3419,7 +3275,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="I26" s="36" t="inlineStr"/>
+      <c r="I26" s="36" t="n"/>
       <c r="J26" s="37" t="inlineStr"/>
     </row>
     <row r="27" ht="115" customHeight="1">
@@ -3463,7 +3319,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="I27" s="36" t="inlineStr"/>
+      <c r="I27" s="36" t="n"/>
       <c r="J27" s="37" t="inlineStr"/>
     </row>
     <row r="28" ht="115" customHeight="1">
@@ -3507,7 +3363,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="I28" s="36" t="inlineStr"/>
+      <c r="I28" s="36" t="n"/>
       <c r="J28" s="37" t="inlineStr"/>
     </row>
     <row r="29" ht="115" customHeight="1">
@@ -3551,7 +3407,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="I29" s="36" t="inlineStr"/>
+      <c r="I29" s="36" t="n"/>
       <c r="J29" s="37" t="inlineStr"/>
     </row>
     <row r="30" ht="115" customHeight="1">
@@ -3595,7 +3451,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="I30" s="36" t="inlineStr"/>
+      <c r="I30" s="36" t="n"/>
       <c r="J30" s="37" t="inlineStr"/>
     </row>
     <row r="31" ht="115" customHeight="1">
@@ -3639,7 +3495,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="I31" s="36" t="inlineStr"/>
+      <c r="I31" s="36" t="n"/>
       <c r="J31" s="37" t="inlineStr"/>
     </row>
     <row r="32" ht="115" customHeight="1">
@@ -3683,7 +3539,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="I32" s="36" t="inlineStr"/>
+      <c r="I32" s="36" t="n"/>
       <c r="J32" s="37" t="inlineStr"/>
     </row>
     <row r="33" ht="115" customHeight="1">
@@ -3727,7 +3583,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="I33" s="36" t="inlineStr"/>
+      <c r="I33" s="36" t="n"/>
       <c r="J33" s="37" t="inlineStr"/>
     </row>
     <row r="34" ht="115" customHeight="1">
@@ -3771,7 +3627,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="I34" s="36" t="inlineStr"/>
+      <c r="I34" s="36" t="n"/>
       <c r="J34" s="37" t="inlineStr"/>
     </row>
     <row r="35" ht="115" customHeight="1">
@@ -3815,7 +3671,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="I35" s="36" t="inlineStr"/>
+      <c r="I35" s="36" t="n"/>
       <c r="J35" s="37" t="inlineStr"/>
     </row>
     <row r="36" ht="115" customHeight="1">
@@ -3859,7 +3715,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="I36" s="36" t="inlineStr"/>
+      <c r="I36" s="36" t="n"/>
       <c r="J36" s="37" t="inlineStr"/>
     </row>
     <row r="37" ht="115" customHeight="1">
@@ -3903,7 +3759,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="I37" s="36" t="inlineStr"/>
+      <c r="I37" s="36" t="n"/>
       <c r="J37" s="37" t="inlineStr"/>
     </row>
     <row r="38" ht="115" customHeight="1">
@@ -3947,7 +3803,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="I38" s="36" t="inlineStr"/>
+      <c r="I38" s="36" t="n"/>
       <c r="J38" s="37" t="inlineStr"/>
     </row>
     <row r="39" ht="115" customHeight="1">
@@ -3991,7 +3847,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="I39" s="36" t="inlineStr"/>
+      <c r="I39" s="36" t="n"/>
       <c r="J39" s="37" t="inlineStr"/>
     </row>
     <row r="40" ht="115" customHeight="1">
@@ -4035,7 +3891,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="I40" s="36" t="inlineStr"/>
+      <c r="I40" s="36" t="n"/>
       <c r="J40" s="37" t="inlineStr"/>
     </row>
     <row r="41" ht="115" customHeight="1">
@@ -4079,7 +3935,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="I41" s="36" t="inlineStr"/>
+      <c r="I41" s="36" t="n"/>
       <c r="J41" s="37" t="inlineStr"/>
     </row>
     <row r="42" ht="115" customHeight="1">
@@ -4123,7 +3979,7 @@
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="I42" s="36" t="inlineStr"/>
+      <c r="I42" s="36" t="n"/>
       <c r="J42" s="37" t="inlineStr"/>
     </row>
     <row r="43" ht="115" customHeight="1">
@@ -4167,7 +4023,7 @@
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="I43" s="36" t="inlineStr"/>
+      <c r="I43" s="36" t="n"/>
       <c r="J43" s="37" t="inlineStr"/>
     </row>
     <row r="44" ht="115" customHeight="1">
@@ -4211,7 +4067,7 @@
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="I44" s="36" t="inlineStr"/>
+      <c r="I44" s="36" t="n"/>
       <c r="J44" s="37" t="inlineStr"/>
     </row>
     <row r="45" ht="115" customHeight="1">
@@ -4255,7 +4111,7 @@
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="I45" s="36" t="inlineStr"/>
+      <c r="I45" s="36" t="n"/>
       <c r="J45" s="37" t="inlineStr"/>
     </row>
     <row r="46" ht="115" customHeight="1">
@@ -4299,7 +4155,7 @@
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="I46" s="36" t="inlineStr"/>
+      <c r="I46" s="36" t="n"/>
       <c r="J46" s="37" t="inlineStr"/>
     </row>
     <row r="47" ht="115" customHeight="1">
@@ -4343,7 +4199,7 @@
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="I47" s="36" t="inlineStr"/>
+      <c r="I47" s="36" t="n"/>
       <c r="J47" s="37" t="inlineStr"/>
     </row>
     <row r="48" ht="115" customHeight="1">
@@ -4387,7 +4243,7 @@
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="I48" s="36" t="inlineStr"/>
+      <c r="I48" s="36" t="n"/>
       <c r="J48" s="37" t="inlineStr"/>
     </row>
     <row r="49" ht="115" customHeight="1">
@@ -4431,7 +4287,7 @@
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="I49" s="36" t="inlineStr"/>
+      <c r="I49" s="36" t="n"/>
       <c r="J49" s="37" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>